<commit_message>
Se agregan módulos adicionales: ventade pollito/huevos - produc-huevos
</commit_message>
<xml_diff>
--- a/data/excelfiles/venta-pollito.xlsx
+++ b/data/excelfiles/venta-pollito.xlsx
@@ -5,17 +5,17 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\wrodriguez\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://pronaca365-my.sharepoint.com/personal/wrodriguez_pronaca_com/Documents/Documentos/Proyectos Django/ETL_SIP/data/excelfiles/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{F5814135-CAFC-4ADA-AB8B-50FA76D818BF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="19" documentId="8_{F5814135-CAFC-4ADA-AB8B-50FA76D818BF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E4A33046-E674-4F7C-8DA9-41BAA438E5D7}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{1F42961E-A269-4130-9414-D8EEB97BFE39}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{1F42961E-A269-4130-9414-D8EEB97BFE39}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="191028"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2184" uniqueCount="360">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2212" uniqueCount="374">
   <si>
     <t>IRN</t>
   </si>
@@ -1119,6 +1119,48 @@
   </si>
   <si>
     <t>3B3B4FFC-D4B5-F111-89B7-005056892616</t>
+  </si>
+  <si>
+    <t>irn</t>
+  </si>
+  <si>
+    <t>fecha envio</t>
+  </si>
+  <si>
+    <t>cantidad</t>
+  </si>
+  <si>
+    <t>fecha semana</t>
+  </si>
+  <si>
+    <t>Tipo Transaccion</t>
+  </si>
+  <si>
+    <t>no incubadora</t>
+  </si>
+  <si>
+    <t>fecha_carga</t>
+  </si>
+  <si>
+    <t>fecha nacimiento</t>
+  </si>
+  <si>
+    <t>semana nacimiento</t>
+  </si>
+  <si>
+    <t>granja lote</t>
+  </si>
+  <si>
+    <t>Cliente</t>
+  </si>
+  <si>
+    <t>Tipo documento</t>
+  </si>
+  <si>
+    <t>No documento</t>
+  </si>
+  <si>
+    <t>END LINE</t>
   </si>
 </sst>
 </file>
@@ -1126,9 +1168,9 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
-    <numFmt numFmtId="165" formatCode="yyyy\-mm\-dd;@"/>
+    <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd;@"/>
   </numFmts>
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1136,16 +1178,54 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="6">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFD3D3D3"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.59999389629810485"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.59999389629810485"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -1153,14 +1233,63 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFA9A9A9"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFA9A9A9"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFA9A9A9"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFA9A9A9"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="11" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="49" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="2" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="14" fontId="1" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="49" fontId="1" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="1" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="164" fontId="0" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1495,16 +1624,18 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E45E131C-AEBA-45AC-A08D-5F1AC8B12301}">
-  <dimension ref="A1:N311"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:N319"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.453125" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="2" max="2" width="11.5546875" style="2"/>
-    <col min="4" max="4" width="11.5546875" style="2"/>
-    <col min="7" max="8" width="11.5546875" style="2"/>
-    <col min="10" max="10" width="11.5546875" style="2"/>
+    <col min="2" max="2" width="11.54296875" style="2"/>
+    <col min="4" max="4" width="11.54296875" style="2"/>
+    <col min="7" max="8" width="11.54296875" style="2"/>
+    <col min="10" max="10" width="11.54296875" style="2"/>
+    <col min="11" max="11" width="14.08984375" customWidth="1"/>
+    <col min="13" max="13" width="13" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1548,7 +1679,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="2" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>13</v>
       </c>
@@ -1592,7 +1723,7 @@
         <v>5535</v>
       </c>
     </row>
-    <row r="3" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>19</v>
       </c>
@@ -1636,7 +1767,7 @@
         <v>5535</v>
       </c>
     </row>
-    <row r="4" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>20</v>
       </c>
@@ -1680,7 +1811,7 @@
         <v>5535</v>
       </c>
     </row>
-    <row r="5" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>21</v>
       </c>
@@ -1724,7 +1855,7 @@
         <v>5535</v>
       </c>
     </row>
-    <row r="6" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>22</v>
       </c>
@@ -1768,7 +1899,7 @@
         <v>5536</v>
       </c>
     </row>
-    <row r="7" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>24</v>
       </c>
@@ -1812,7 +1943,7 @@
         <v>5536</v>
       </c>
     </row>
-    <row r="8" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>25</v>
       </c>
@@ -1856,7 +1987,7 @@
         <v>5541</v>
       </c>
     </row>
-    <row r="9" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>28</v>
       </c>
@@ -1900,7 +2031,7 @@
         <v>5541</v>
       </c>
     </row>
-    <row r="10" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>29</v>
       </c>
@@ -1944,7 +2075,7 @@
         <v>5541</v>
       </c>
     </row>
-    <row r="11" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>30</v>
       </c>
@@ -1988,7 +2119,7 @@
         <v>5541</v>
       </c>
     </row>
-    <row r="12" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>31</v>
       </c>
@@ -2032,7 +2163,7 @@
         <v>5534</v>
       </c>
     </row>
-    <row r="13" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>35</v>
       </c>
@@ -2076,7 +2207,7 @@
         <v>5534</v>
       </c>
     </row>
-    <row r="14" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
         <v>36</v>
       </c>
@@ -2120,7 +2251,7 @@
         <v>5534</v>
       </c>
     </row>
-    <row r="15" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:14" hidden="1" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
         <v>37</v>
       </c>
@@ -2164,7 +2295,7 @@
         <v>5534</v>
       </c>
     </row>
-    <row r="16" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:14" hidden="1" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
         <v>38</v>
       </c>
@@ -2208,7 +2339,7 @@
         <v>5534</v>
       </c>
     </row>
-    <row r="17" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:14" hidden="1" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
         <v>39</v>
       </c>
@@ -2252,7 +2383,7 @@
         <v>5534</v>
       </c>
     </row>
-    <row r="18" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:14" hidden="1" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
         <v>40</v>
       </c>
@@ -2296,7 +2427,7 @@
         <v>5534</v>
       </c>
     </row>
-    <row r="19" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:14" hidden="1" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
         <v>41</v>
       </c>
@@ -2340,7 +2471,7 @@
         <v>5534</v>
       </c>
     </row>
-    <row r="20" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:14" hidden="1" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
         <v>42</v>
       </c>
@@ -2384,7 +2515,7 @@
         <v>5533</v>
       </c>
     </row>
-    <row r="21" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:14" hidden="1" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
         <v>45</v>
       </c>
@@ -2428,7 +2559,7 @@
         <v>5533</v>
       </c>
     </row>
-    <row r="22" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:14" hidden="1" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
         <v>46</v>
       </c>
@@ -2472,7 +2603,7 @@
         <v>5533</v>
       </c>
     </row>
-    <row r="23" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:14" hidden="1" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
         <v>47</v>
       </c>
@@ -2516,7 +2647,7 @@
         <v>5533</v>
       </c>
     </row>
-    <row r="24" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:14" hidden="1" x14ac:dyDescent="0.35">
       <c r="A24" t="s">
         <v>48</v>
       </c>
@@ -2560,7 +2691,7 @@
         <v>5533</v>
       </c>
     </row>
-    <row r="25" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:14" hidden="1" x14ac:dyDescent="0.35">
       <c r="A25" t="s">
         <v>49</v>
       </c>
@@ -2604,7 +2735,7 @@
         <v>5533</v>
       </c>
     </row>
-    <row r="26" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:14" hidden="1" x14ac:dyDescent="0.35">
       <c r="A26" t="s">
         <v>50</v>
       </c>
@@ -2648,7 +2779,7 @@
         <v>5535</v>
       </c>
     </row>
-    <row r="27" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:14" hidden="1" x14ac:dyDescent="0.35">
       <c r="A27" t="s">
         <v>52</v>
       </c>
@@ -2692,7 +2823,7 @@
         <v>5535</v>
       </c>
     </row>
-    <row r="28" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:14" hidden="1" x14ac:dyDescent="0.35">
       <c r="A28" t="s">
         <v>53</v>
       </c>
@@ -2736,7 +2867,7 @@
         <v>5535</v>
       </c>
     </row>
-    <row r="29" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:14" hidden="1" x14ac:dyDescent="0.35">
       <c r="A29" t="s">
         <v>54</v>
       </c>
@@ -2780,7 +2911,7 @@
         <v>5535</v>
       </c>
     </row>
-    <row r="30" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:14" hidden="1" x14ac:dyDescent="0.35">
       <c r="A30" t="s">
         <v>55</v>
       </c>
@@ -2824,7 +2955,7 @@
         <v>5535</v>
       </c>
     </row>
-    <row r="31" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:14" hidden="1" x14ac:dyDescent="0.35">
       <c r="A31" t="s">
         <v>56</v>
       </c>
@@ -2868,7 +2999,7 @@
         <v>5535</v>
       </c>
     </row>
-    <row r="32" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:14" hidden="1" x14ac:dyDescent="0.35">
       <c r="A32" t="s">
         <v>57</v>
       </c>
@@ -2912,7 +3043,7 @@
         <v>5539</v>
       </c>
     </row>
-    <row r="33" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:14" hidden="1" x14ac:dyDescent="0.35">
       <c r="A33" t="s">
         <v>60</v>
       </c>
@@ -2956,7 +3087,7 @@
         <v>5539</v>
       </c>
     </row>
-    <row r="34" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:14" hidden="1" x14ac:dyDescent="0.35">
       <c r="A34" t="s">
         <v>61</v>
       </c>
@@ -3000,7 +3131,7 @@
         <v>5539</v>
       </c>
     </row>
-    <row r="35" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:14" hidden="1" x14ac:dyDescent="0.35">
       <c r="A35" t="s">
         <v>62</v>
       </c>
@@ -3044,7 +3175,7 @@
         <v>5539</v>
       </c>
     </row>
-    <row r="36" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:14" hidden="1" x14ac:dyDescent="0.35">
       <c r="A36" t="s">
         <v>63</v>
       </c>
@@ -3088,7 +3219,7 @@
         <v>5539</v>
       </c>
     </row>
-    <row r="37" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:14" hidden="1" x14ac:dyDescent="0.35">
       <c r="A37" t="s">
         <v>64</v>
       </c>
@@ -3132,7 +3263,7 @@
         <v>5539</v>
       </c>
     </row>
-    <row r="38" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:14" hidden="1" x14ac:dyDescent="0.35">
       <c r="A38" t="s">
         <v>65</v>
       </c>
@@ -3176,7 +3307,7 @@
         <v>5536</v>
       </c>
     </row>
-    <row r="39" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:14" hidden="1" x14ac:dyDescent="0.35">
       <c r="A39" t="s">
         <v>66</v>
       </c>
@@ -3220,7 +3351,7 @@
         <v>5536</v>
       </c>
     </row>
-    <row r="40" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:14" hidden="1" x14ac:dyDescent="0.35">
       <c r="A40" t="s">
         <v>67</v>
       </c>
@@ -3264,7 +3395,7 @@
         <v>5536</v>
       </c>
     </row>
-    <row r="41" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:14" hidden="1" x14ac:dyDescent="0.35">
       <c r="A41" t="s">
         <v>68</v>
       </c>
@@ -3308,7 +3439,7 @@
         <v>5536</v>
       </c>
     </row>
-    <row r="42" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:14" hidden="1" x14ac:dyDescent="0.35">
       <c r="A42" t="s">
         <v>69</v>
       </c>
@@ -3352,7 +3483,7 @@
         <v>5536</v>
       </c>
     </row>
-    <row r="43" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:14" hidden="1" x14ac:dyDescent="0.35">
       <c r="A43" t="s">
         <v>71</v>
       </c>
@@ -3396,7 +3527,7 @@
         <v>5536</v>
       </c>
     </row>
-    <row r="44" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:14" hidden="1" x14ac:dyDescent="0.35">
       <c r="A44" t="s">
         <v>72</v>
       </c>
@@ -3440,7 +3571,7 @@
         <v>5536</v>
       </c>
     </row>
-    <row r="45" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:14" hidden="1" x14ac:dyDescent="0.35">
       <c r="A45" t="s">
         <v>73</v>
       </c>
@@ -3484,7 +3615,7 @@
         <v>5536</v>
       </c>
     </row>
-    <row r="46" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:14" hidden="1" x14ac:dyDescent="0.35">
       <c r="A46" t="s">
         <v>74</v>
       </c>
@@ -3528,7 +3659,7 @@
         <v>5536</v>
       </c>
     </row>
-    <row r="47" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:14" hidden="1" x14ac:dyDescent="0.35">
       <c r="A47" t="s">
         <v>75</v>
       </c>
@@ -3572,7 +3703,7 @@
         <v>5536</v>
       </c>
     </row>
-    <row r="48" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:14" hidden="1" x14ac:dyDescent="0.35">
       <c r="A48" t="s">
         <v>76</v>
       </c>
@@ -3616,7 +3747,7 @@
         <v>5536</v>
       </c>
     </row>
-    <row r="49" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:14" hidden="1" x14ac:dyDescent="0.35">
       <c r="A49" t="s">
         <v>77</v>
       </c>
@@ -3660,7 +3791,7 @@
         <v>5536</v>
       </c>
     </row>
-    <row r="50" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:14" hidden="1" x14ac:dyDescent="0.35">
       <c r="A50" t="s">
         <v>78</v>
       </c>
@@ -3704,7 +3835,7 @@
         <v>5532</v>
       </c>
     </row>
-    <row r="51" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:14" hidden="1" x14ac:dyDescent="0.35">
       <c r="A51" t="s">
         <v>80</v>
       </c>
@@ -3748,7 +3879,7 @@
         <v>5532</v>
       </c>
     </row>
-    <row r="52" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:14" hidden="1" x14ac:dyDescent="0.35">
       <c r="A52" t="s">
         <v>81</v>
       </c>
@@ -3792,7 +3923,7 @@
         <v>5532</v>
       </c>
     </row>
-    <row r="53" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:14" hidden="1" x14ac:dyDescent="0.35">
       <c r="A53" t="s">
         <v>82</v>
       </c>
@@ -3836,7 +3967,7 @@
         <v>5532</v>
       </c>
     </row>
-    <row r="54" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:14" hidden="1" x14ac:dyDescent="0.35">
       <c r="A54" t="s">
         <v>83</v>
       </c>
@@ -3880,7 +4011,7 @@
         <v>5532</v>
       </c>
     </row>
-    <row r="55" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:14" hidden="1" x14ac:dyDescent="0.35">
       <c r="A55" t="s">
         <v>84</v>
       </c>
@@ -3924,7 +4055,7 @@
         <v>5532</v>
       </c>
     </row>
-    <row r="56" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:14" hidden="1" x14ac:dyDescent="0.35">
       <c r="A56" t="s">
         <v>85</v>
       </c>
@@ -3968,7 +4099,7 @@
         <v>5532</v>
       </c>
     </row>
-    <row r="57" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:14" hidden="1" x14ac:dyDescent="0.35">
       <c r="A57" s="1" t="s">
         <v>86</v>
       </c>
@@ -4012,7 +4143,7 @@
         <v>5532</v>
       </c>
     </row>
-    <row r="58" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="58" spans="1:14" hidden="1" x14ac:dyDescent="0.35">
       <c r="A58" t="s">
         <v>87</v>
       </c>
@@ -4056,7 +4187,7 @@
         <v>5532</v>
       </c>
     </row>
-    <row r="59" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="59" spans="1:14" hidden="1" x14ac:dyDescent="0.35">
       <c r="A59" t="s">
         <v>88</v>
       </c>
@@ -4100,7 +4231,7 @@
         <v>5532</v>
       </c>
     </row>
-    <row r="60" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="60" spans="1:14" hidden="1" x14ac:dyDescent="0.35">
       <c r="A60" t="s">
         <v>89</v>
       </c>
@@ -4144,7 +4275,7 @@
         <v>5535</v>
       </c>
     </row>
-    <row r="61" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="61" spans="1:14" hidden="1" x14ac:dyDescent="0.35">
       <c r="A61" t="s">
         <v>90</v>
       </c>
@@ -4188,7 +4319,7 @@
         <v>5535</v>
       </c>
     </row>
-    <row r="62" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="62" spans="1:14" hidden="1" x14ac:dyDescent="0.35">
       <c r="A62" t="s">
         <v>91</v>
       </c>
@@ -4232,7 +4363,7 @@
         <v>5535</v>
       </c>
     </row>
-    <row r="63" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="63" spans="1:14" hidden="1" x14ac:dyDescent="0.35">
       <c r="A63" t="s">
         <v>92</v>
       </c>
@@ -4276,7 +4407,7 @@
         <v>5535</v>
       </c>
     </row>
-    <row r="64" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="64" spans="1:14" hidden="1" x14ac:dyDescent="0.35">
       <c r="A64" t="s">
         <v>93</v>
       </c>
@@ -4320,7 +4451,7 @@
         <v>5535</v>
       </c>
     </row>
-    <row r="65" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="65" spans="1:14" hidden="1" x14ac:dyDescent="0.35">
       <c r="A65" t="s">
         <v>94</v>
       </c>
@@ -4364,7 +4495,7 @@
         <v>5535</v>
       </c>
     </row>
-    <row r="66" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="66" spans="1:14" hidden="1" x14ac:dyDescent="0.35">
       <c r="A66" t="s">
         <v>95</v>
       </c>
@@ -4408,7 +4539,7 @@
         <v>5541</v>
       </c>
     </row>
-    <row r="67" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="67" spans="1:14" hidden="1" x14ac:dyDescent="0.35">
       <c r="A67" t="s">
         <v>97</v>
       </c>
@@ -4452,7 +4583,7 @@
         <v>5541</v>
       </c>
     </row>
-    <row r="68" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="68" spans="1:14" hidden="1" x14ac:dyDescent="0.35">
       <c r="A68" t="s">
         <v>98</v>
       </c>
@@ -4496,7 +4627,7 @@
         <v>5542</v>
       </c>
     </row>
-    <row r="69" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="69" spans="1:14" hidden="1" x14ac:dyDescent="0.35">
       <c r="A69" t="s">
         <v>101</v>
       </c>
@@ -4540,7 +4671,7 @@
         <v>5542</v>
       </c>
     </row>
-    <row r="70" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="70" spans="1:14" hidden="1" x14ac:dyDescent="0.35">
       <c r="A70" t="s">
         <v>102</v>
       </c>
@@ -4584,7 +4715,7 @@
         <v>5542</v>
       </c>
     </row>
-    <row r="71" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="71" spans="1:14" hidden="1" x14ac:dyDescent="0.35">
       <c r="A71" t="s">
         <v>103</v>
       </c>
@@ -4628,7 +4759,7 @@
         <v>5543</v>
       </c>
     </row>
-    <row r="72" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="72" spans="1:14" hidden="1" x14ac:dyDescent="0.35">
       <c r="A72" t="s">
         <v>105</v>
       </c>
@@ -4672,7 +4803,7 @@
         <v>5543</v>
       </c>
     </row>
-    <row r="73" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="73" spans="1:14" hidden="1" x14ac:dyDescent="0.35">
       <c r="A73" t="s">
         <v>106</v>
       </c>
@@ -4716,7 +4847,7 @@
         <v>5543</v>
       </c>
     </row>
-    <row r="74" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="74" spans="1:14" hidden="1" x14ac:dyDescent="0.35">
       <c r="A74" t="s">
         <v>107</v>
       </c>
@@ -4760,7 +4891,7 @@
         <v>5543</v>
       </c>
     </row>
-    <row r="75" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="75" spans="1:14" hidden="1" x14ac:dyDescent="0.35">
       <c r="A75" t="s">
         <v>108</v>
       </c>
@@ -4804,7 +4935,7 @@
         <v>5536</v>
       </c>
     </row>
-    <row r="76" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="76" spans="1:14" hidden="1" x14ac:dyDescent="0.35">
       <c r="A76" t="s">
         <v>109</v>
       </c>
@@ -4848,7 +4979,7 @@
         <v>5536</v>
       </c>
     </row>
-    <row r="77" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="77" spans="1:14" hidden="1" x14ac:dyDescent="0.35">
       <c r="A77" t="s">
         <v>110</v>
       </c>
@@ -4892,7 +5023,7 @@
         <v>5536</v>
       </c>
     </row>
-    <row r="78" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="78" spans="1:14" hidden="1" x14ac:dyDescent="0.35">
       <c r="A78" t="s">
         <v>111</v>
       </c>
@@ -4936,7 +5067,7 @@
         <v>5536</v>
       </c>
     </row>
-    <row r="79" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="79" spans="1:14" hidden="1" x14ac:dyDescent="0.35">
       <c r="A79" t="s">
         <v>112</v>
       </c>
@@ -4980,7 +5111,7 @@
         <v>5540</v>
       </c>
     </row>
-    <row r="80" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="80" spans="1:14" hidden="1" x14ac:dyDescent="0.35">
       <c r="A80" t="s">
         <v>114</v>
       </c>
@@ -5024,7 +5155,7 @@
         <v>5540</v>
       </c>
     </row>
-    <row r="81" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="81" spans="1:14" hidden="1" x14ac:dyDescent="0.35">
       <c r="A81" t="s">
         <v>115</v>
       </c>
@@ -5068,7 +5199,7 @@
         <v>5540</v>
       </c>
     </row>
-    <row r="82" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="82" spans="1:14" hidden="1" x14ac:dyDescent="0.35">
       <c r="A82" t="s">
         <v>116</v>
       </c>
@@ -5112,7 +5243,7 @@
         <v>5540</v>
       </c>
     </row>
-    <row r="83" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="83" spans="1:14" hidden="1" x14ac:dyDescent="0.35">
       <c r="A83" t="s">
         <v>117</v>
       </c>
@@ -5156,7 +5287,7 @@
         <v>5540</v>
       </c>
     </row>
-    <row r="84" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="84" spans="1:14" hidden="1" x14ac:dyDescent="0.35">
       <c r="A84" t="s">
         <v>118</v>
       </c>
@@ -5200,7 +5331,7 @@
         <v>5540</v>
       </c>
     </row>
-    <row r="85" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="85" spans="1:14" hidden="1" x14ac:dyDescent="0.35">
       <c r="A85" t="s">
         <v>119</v>
       </c>
@@ -5244,7 +5375,7 @@
         <v>5540</v>
       </c>
     </row>
-    <row r="86" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="86" spans="1:14" hidden="1" x14ac:dyDescent="0.35">
       <c r="A86" t="s">
         <v>120</v>
       </c>
@@ -5288,7 +5419,7 @@
         <v>5540</v>
       </c>
     </row>
-    <row r="87" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="87" spans="1:14" hidden="1" x14ac:dyDescent="0.35">
       <c r="A87" t="s">
         <v>121</v>
       </c>
@@ -5332,7 +5463,7 @@
         <v>5535</v>
       </c>
     </row>
-    <row r="88" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="88" spans="1:14" hidden="1" x14ac:dyDescent="0.35">
       <c r="A88" t="s">
         <v>122</v>
       </c>
@@ -5376,7 +5507,7 @@
         <v>5535</v>
       </c>
     </row>
-    <row r="89" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="89" spans="1:14" hidden="1" x14ac:dyDescent="0.35">
       <c r="A89" t="s">
         <v>123</v>
       </c>
@@ -5420,7 +5551,7 @@
         <v>5535</v>
       </c>
     </row>
-    <row r="90" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="90" spans="1:14" hidden="1" x14ac:dyDescent="0.35">
       <c r="A90" t="s">
         <v>124</v>
       </c>
@@ -5464,7 +5595,7 @@
         <v>5535</v>
       </c>
     </row>
-    <row r="91" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="91" spans="1:14" hidden="1" x14ac:dyDescent="0.35">
       <c r="A91" t="s">
         <v>125</v>
       </c>
@@ -5508,7 +5639,7 @@
         <v>5535</v>
       </c>
     </row>
-    <row r="92" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="92" spans="1:14" hidden="1" x14ac:dyDescent="0.35">
       <c r="A92" t="s">
         <v>126</v>
       </c>
@@ -5552,7 +5683,7 @@
         <v>5535</v>
       </c>
     </row>
-    <row r="93" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="93" spans="1:14" hidden="1" x14ac:dyDescent="0.35">
       <c r="A93" t="s">
         <v>128</v>
       </c>
@@ -5596,7 +5727,7 @@
         <v>5535</v>
       </c>
     </row>
-    <row r="94" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="94" spans="1:14" hidden="1" x14ac:dyDescent="0.35">
       <c r="A94" t="s">
         <v>129</v>
       </c>
@@ -5640,7 +5771,7 @@
         <v>5535</v>
       </c>
     </row>
-    <row r="95" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="95" spans="1:14" hidden="1" x14ac:dyDescent="0.35">
       <c r="A95" t="s">
         <v>130</v>
       </c>
@@ -5684,7 +5815,7 @@
         <v>5535</v>
       </c>
     </row>
-    <row r="96" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="96" spans="1:14" hidden="1" x14ac:dyDescent="0.35">
       <c r="A96" t="s">
         <v>131</v>
       </c>
@@ -5728,7 +5859,7 @@
         <v>5536</v>
       </c>
     </row>
-    <row r="97" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="97" spans="1:14" hidden="1" x14ac:dyDescent="0.35">
       <c r="A97" t="s">
         <v>132</v>
       </c>
@@ -5772,7 +5903,7 @@
         <v>5536</v>
       </c>
     </row>
-    <row r="98" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="98" spans="1:14" hidden="1" x14ac:dyDescent="0.35">
       <c r="A98" t="s">
         <v>133</v>
       </c>
@@ -5816,7 +5947,7 @@
         <v>5540</v>
       </c>
     </row>
-    <row r="99" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="99" spans="1:14" hidden="1" x14ac:dyDescent="0.35">
       <c r="A99" t="s">
         <v>134</v>
       </c>
@@ -5860,7 +5991,7 @@
         <v>5540</v>
       </c>
     </row>
-    <row r="100" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="100" spans="1:14" hidden="1" x14ac:dyDescent="0.35">
       <c r="A100" t="s">
         <v>135</v>
       </c>
@@ -5904,7 +6035,7 @@
         <v>5540</v>
       </c>
     </row>
-    <row r="101" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="101" spans="1:14" hidden="1" x14ac:dyDescent="0.35">
       <c r="A101" t="s">
         <v>136</v>
       </c>
@@ -5948,7 +6079,7 @@
         <v>5540</v>
       </c>
     </row>
-    <row r="102" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="102" spans="1:14" hidden="1" x14ac:dyDescent="0.35">
       <c r="A102" t="s">
         <v>137</v>
       </c>
@@ -5992,7 +6123,7 @@
         <v>5540</v>
       </c>
     </row>
-    <row r="103" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="103" spans="1:14" hidden="1" x14ac:dyDescent="0.35">
       <c r="A103" t="s">
         <v>138</v>
       </c>
@@ -6036,7 +6167,7 @@
         <v>5540</v>
       </c>
     </row>
-    <row r="104" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="104" spans="1:14" hidden="1" x14ac:dyDescent="0.35">
       <c r="A104" t="s">
         <v>139</v>
       </c>
@@ -6080,7 +6211,7 @@
         <v>5541</v>
       </c>
     </row>
-    <row r="105" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="105" spans="1:14" hidden="1" x14ac:dyDescent="0.35">
       <c r="A105" t="s">
         <v>140</v>
       </c>
@@ -6124,7 +6255,7 @@
         <v>5541</v>
       </c>
     </row>
-    <row r="106" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="106" spans="1:14" hidden="1" x14ac:dyDescent="0.35">
       <c r="A106" t="s">
         <v>141</v>
       </c>
@@ -6168,7 +6299,7 @@
         <v>5541</v>
       </c>
     </row>
-    <row r="107" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="107" spans="1:14" hidden="1" x14ac:dyDescent="0.35">
       <c r="A107" t="s">
         <v>142</v>
       </c>
@@ -6212,7 +6343,7 @@
         <v>5541</v>
       </c>
     </row>
-    <row r="108" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="108" spans="1:14" hidden="1" x14ac:dyDescent="0.35">
       <c r="A108" t="s">
         <v>143</v>
       </c>
@@ -6256,7 +6387,7 @@
         <v>5543</v>
       </c>
     </row>
-    <row r="109" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="109" spans="1:14" hidden="1" x14ac:dyDescent="0.35">
       <c r="A109" t="s">
         <v>145</v>
       </c>
@@ -6300,7 +6431,7 @@
         <v>5543</v>
       </c>
     </row>
-    <row r="110" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="110" spans="1:14" hidden="1" x14ac:dyDescent="0.35">
       <c r="A110" t="s">
         <v>146</v>
       </c>
@@ -6344,7 +6475,7 @@
         <v>5543</v>
       </c>
     </row>
-    <row r="111" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="111" spans="1:14" hidden="1" x14ac:dyDescent="0.35">
       <c r="A111" t="s">
         <v>147</v>
       </c>
@@ -6388,7 +6519,7 @@
         <v>5543</v>
       </c>
     </row>
-    <row r="112" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="112" spans="1:14" hidden="1" x14ac:dyDescent="0.35">
       <c r="A112" t="s">
         <v>148</v>
       </c>
@@ -6432,7 +6563,7 @@
         <v>5543</v>
       </c>
     </row>
-    <row r="113" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="113" spans="1:14" hidden="1" x14ac:dyDescent="0.35">
       <c r="A113" t="s">
         <v>149</v>
       </c>
@@ -6476,7 +6607,7 @@
         <v>5543</v>
       </c>
     </row>
-    <row r="114" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="114" spans="1:14" hidden="1" x14ac:dyDescent="0.35">
       <c r="A114" t="s">
         <v>150</v>
       </c>
@@ -6520,7 +6651,7 @@
         <v>5536</v>
       </c>
     </row>
-    <row r="115" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="115" spans="1:14" hidden="1" x14ac:dyDescent="0.35">
       <c r="A115" t="s">
         <v>151</v>
       </c>
@@ -6564,7 +6695,7 @@
         <v>5536</v>
       </c>
     </row>
-    <row r="116" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="116" spans="1:14" hidden="1" x14ac:dyDescent="0.35">
       <c r="A116" t="s">
         <v>152</v>
       </c>
@@ -6608,7 +6739,7 @@
         <v>5540</v>
       </c>
     </row>
-    <row r="117" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="117" spans="1:14" hidden="1" x14ac:dyDescent="0.35">
       <c r="A117" t="s">
         <v>153</v>
       </c>
@@ -6652,7 +6783,7 @@
         <v>5540</v>
       </c>
     </row>
-    <row r="118" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="118" spans="1:14" hidden="1" x14ac:dyDescent="0.35">
       <c r="A118" t="s">
         <v>154</v>
       </c>
@@ -6696,7 +6827,7 @@
         <v>5540</v>
       </c>
     </row>
-    <row r="119" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="119" spans="1:14" hidden="1" x14ac:dyDescent="0.35">
       <c r="A119" t="s">
         <v>155</v>
       </c>
@@ -6740,7 +6871,7 @@
         <v>5540</v>
       </c>
     </row>
-    <row r="120" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="120" spans="1:14" hidden="1" x14ac:dyDescent="0.35">
       <c r="A120" t="s">
         <v>156</v>
       </c>
@@ -6784,7 +6915,7 @@
         <v>5540</v>
       </c>
     </row>
-    <row r="121" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="121" spans="1:14" hidden="1" x14ac:dyDescent="0.35">
       <c r="A121" t="s">
         <v>157</v>
       </c>
@@ -6828,7 +6959,7 @@
         <v>5540</v>
       </c>
     </row>
-    <row r="122" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="122" spans="1:14" hidden="1" x14ac:dyDescent="0.35">
       <c r="A122" t="s">
         <v>158</v>
       </c>
@@ -6872,7 +7003,7 @@
         <v>5535</v>
       </c>
     </row>
-    <row r="123" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="123" spans="1:14" hidden="1" x14ac:dyDescent="0.35">
       <c r="A123" t="s">
         <v>159</v>
       </c>
@@ -6916,7 +7047,7 @@
         <v>5535</v>
       </c>
     </row>
-    <row r="124" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="124" spans="1:14" hidden="1" x14ac:dyDescent="0.35">
       <c r="A124" t="s">
         <v>160</v>
       </c>
@@ -6960,7 +7091,7 @@
         <v>5535</v>
       </c>
     </row>
-    <row r="125" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="125" spans="1:14" hidden="1" x14ac:dyDescent="0.35">
       <c r="A125" t="s">
         <v>161</v>
       </c>
@@ -7004,7 +7135,7 @@
         <v>5535</v>
       </c>
     </row>
-    <row r="126" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="126" spans="1:14" hidden="1" x14ac:dyDescent="0.35">
       <c r="A126" t="s">
         <v>162</v>
       </c>
@@ -7048,7 +7179,7 @@
         <v>5535</v>
       </c>
     </row>
-    <row r="127" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="127" spans="1:14" hidden="1" x14ac:dyDescent="0.35">
       <c r="A127" t="s">
         <v>163</v>
       </c>
@@ -7092,7 +7223,7 @@
         <v>5535</v>
       </c>
     </row>
-    <row r="128" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="128" spans="1:14" hidden="1" x14ac:dyDescent="0.35">
       <c r="A128" t="s">
         <v>164</v>
       </c>
@@ -7136,7 +7267,7 @@
         <v>5538</v>
       </c>
     </row>
-    <row r="129" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="129" spans="1:14" hidden="1" x14ac:dyDescent="0.35">
       <c r="A129" t="s">
         <v>167</v>
       </c>
@@ -7180,7 +7311,7 @@
         <v>5531</v>
       </c>
     </row>
-    <row r="130" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="130" spans="1:14" hidden="1" x14ac:dyDescent="0.35">
       <c r="A130" t="s">
         <v>169</v>
       </c>
@@ -7224,7 +7355,7 @@
         <v>5539</v>
       </c>
     </row>
-    <row r="131" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="131" spans="1:14" hidden="1" x14ac:dyDescent="0.35">
       <c r="A131" t="s">
         <v>171</v>
       </c>
@@ -7268,7 +7399,7 @@
         <v>5539</v>
       </c>
     </row>
-    <row r="132" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="132" spans="1:14" hidden="1" x14ac:dyDescent="0.35">
       <c r="A132" t="s">
         <v>172</v>
       </c>
@@ -7312,7 +7443,7 @@
         <v>5539</v>
       </c>
     </row>
-    <row r="133" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="133" spans="1:14" hidden="1" x14ac:dyDescent="0.35">
       <c r="A133" t="s">
         <v>173</v>
       </c>
@@ -7356,7 +7487,7 @@
         <v>5539</v>
       </c>
     </row>
-    <row r="134" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="134" spans="1:14" hidden="1" x14ac:dyDescent="0.35">
       <c r="A134" t="s">
         <v>174</v>
       </c>
@@ -7400,7 +7531,7 @@
         <v>5539</v>
       </c>
     </row>
-    <row r="135" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="135" spans="1:14" hidden="1" x14ac:dyDescent="0.35">
       <c r="A135" t="s">
         <v>175</v>
       </c>
@@ -7444,7 +7575,7 @@
         <v>5539</v>
       </c>
     </row>
-    <row r="136" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="136" spans="1:14" hidden="1" x14ac:dyDescent="0.35">
       <c r="A136" t="s">
         <v>176</v>
       </c>
@@ -7488,7 +7619,7 @@
         <v>5539</v>
       </c>
     </row>
-    <row r="137" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="137" spans="1:14" hidden="1" x14ac:dyDescent="0.35">
       <c r="A137" t="s">
         <v>177</v>
       </c>
@@ -7532,7 +7663,7 @@
         <v>5539</v>
       </c>
     </row>
-    <row r="138" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="138" spans="1:14" hidden="1" x14ac:dyDescent="0.35">
       <c r="A138" t="s">
         <v>178</v>
       </c>
@@ -7576,7 +7707,7 @@
         <v>5536</v>
       </c>
     </row>
-    <row r="139" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="139" spans="1:14" hidden="1" x14ac:dyDescent="0.35">
       <c r="A139" t="s">
         <v>179</v>
       </c>
@@ -7620,7 +7751,7 @@
         <v>5536</v>
       </c>
     </row>
-    <row r="140" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="140" spans="1:14" hidden="1" x14ac:dyDescent="0.35">
       <c r="A140" t="s">
         <v>180</v>
       </c>
@@ -7664,7 +7795,7 @@
         <v>5536</v>
       </c>
     </row>
-    <row r="141" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="141" spans="1:14" hidden="1" x14ac:dyDescent="0.35">
       <c r="A141" t="s">
         <v>181</v>
       </c>
@@ -7708,7 +7839,7 @@
         <v>5536</v>
       </c>
     </row>
-    <row r="142" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="142" spans="1:14" hidden="1" x14ac:dyDescent="0.35">
       <c r="A142" t="s">
         <v>182</v>
       </c>
@@ -7752,7 +7883,7 @@
         <v>5536</v>
       </c>
     </row>
-    <row r="143" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="143" spans="1:14" hidden="1" x14ac:dyDescent="0.35">
       <c r="A143" t="s">
         <v>183</v>
       </c>
@@ -7796,7 +7927,7 @@
         <v>5536</v>
       </c>
     </row>
-    <row r="144" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="144" spans="1:14" hidden="1" x14ac:dyDescent="0.35">
       <c r="A144" t="s">
         <v>184</v>
       </c>
@@ -7840,7 +7971,7 @@
         <v>5535</v>
       </c>
     </row>
-    <row r="145" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="145" spans="1:14" hidden="1" x14ac:dyDescent="0.35">
       <c r="A145" t="s">
         <v>185</v>
       </c>
@@ -7884,7 +8015,7 @@
         <v>5535</v>
       </c>
     </row>
-    <row r="146" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="146" spans="1:14" hidden="1" x14ac:dyDescent="0.35">
       <c r="A146" t="s">
         <v>186</v>
       </c>
@@ -7928,7 +8059,7 @@
         <v>5535</v>
       </c>
     </row>
-    <row r="147" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="147" spans="1:14" hidden="1" x14ac:dyDescent="0.35">
       <c r="A147" t="s">
         <v>187</v>
       </c>
@@ -7972,7 +8103,7 @@
         <v>5535</v>
       </c>
     </row>
-    <row r="148" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="148" spans="1:14" hidden="1" x14ac:dyDescent="0.35">
       <c r="A148" t="s">
         <v>188</v>
       </c>
@@ -8016,7 +8147,7 @@
         <v>5535</v>
       </c>
     </row>
-    <row r="149" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="149" spans="1:14" hidden="1" x14ac:dyDescent="0.35">
       <c r="A149" t="s">
         <v>189</v>
       </c>
@@ -8060,7 +8191,7 @@
         <v>5535</v>
       </c>
     </row>
-    <row r="150" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="150" spans="1:14" hidden="1" x14ac:dyDescent="0.35">
       <c r="A150" t="s">
         <v>190</v>
       </c>
@@ -8104,7 +8235,7 @@
         <v>5535</v>
       </c>
     </row>
-    <row r="151" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="151" spans="1:14" hidden="1" x14ac:dyDescent="0.35">
       <c r="A151" t="s">
         <v>192</v>
       </c>
@@ -8148,7 +8279,7 @@
         <v>5535</v>
       </c>
     </row>
-    <row r="152" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="152" spans="1:14" hidden="1" x14ac:dyDescent="0.35">
       <c r="A152" t="s">
         <v>193</v>
       </c>
@@ -8192,7 +8323,7 @@
         <v>5535</v>
       </c>
     </row>
-    <row r="153" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="153" spans="1:14" hidden="1" x14ac:dyDescent="0.35">
       <c r="A153" t="s">
         <v>194</v>
       </c>
@@ -8236,7 +8367,7 @@
         <v>5535</v>
       </c>
     </row>
-    <row r="154" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="154" spans="1:14" hidden="1" x14ac:dyDescent="0.35">
       <c r="A154" t="s">
         <v>195</v>
       </c>
@@ -8280,7 +8411,7 @@
         <v>5541</v>
       </c>
     </row>
-    <row r="155" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="155" spans="1:14" hidden="1" x14ac:dyDescent="0.35">
       <c r="A155" t="s">
         <v>196</v>
       </c>
@@ -8324,7 +8455,7 @@
         <v>5541</v>
       </c>
     </row>
-    <row r="156" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="156" spans="1:14" hidden="1" x14ac:dyDescent="0.35">
       <c r="A156" t="s">
         <v>197</v>
       </c>
@@ -8368,7 +8499,7 @@
         <v>5536</v>
       </c>
     </row>
-    <row r="157" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="157" spans="1:14" hidden="1" x14ac:dyDescent="0.35">
       <c r="A157" t="s">
         <v>198</v>
       </c>
@@ -8412,7 +8543,7 @@
         <v>5536</v>
       </c>
     </row>
-    <row r="158" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="158" spans="1:14" hidden="1" x14ac:dyDescent="0.35">
       <c r="A158" t="s">
         <v>199</v>
       </c>
@@ -8456,7 +8587,7 @@
         <v>5536</v>
       </c>
     </row>
-    <row r="159" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="159" spans="1:14" hidden="1" x14ac:dyDescent="0.35">
       <c r="A159" t="s">
         <v>200</v>
       </c>
@@ -8500,7 +8631,7 @@
         <v>5536</v>
       </c>
     </row>
-    <row r="160" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="160" spans="1:14" hidden="1" x14ac:dyDescent="0.35">
       <c r="A160" t="s">
         <v>201</v>
       </c>
@@ -8544,7 +8675,7 @@
         <v>5541</v>
       </c>
     </row>
-    <row r="161" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="161" spans="1:14" hidden="1" x14ac:dyDescent="0.35">
       <c r="A161" t="s">
         <v>203</v>
       </c>
@@ -8588,7 +8719,7 @@
         <v>5541</v>
       </c>
     </row>
-    <row r="162" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="162" spans="1:14" hidden="1" x14ac:dyDescent="0.35">
       <c r="A162" t="s">
         <v>204</v>
       </c>
@@ -8632,7 +8763,7 @@
         <v>5541</v>
       </c>
     </row>
-    <row r="163" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="163" spans="1:14" hidden="1" x14ac:dyDescent="0.35">
       <c r="A163" t="s">
         <v>205</v>
       </c>
@@ -8676,7 +8807,7 @@
         <v>5541</v>
       </c>
     </row>
-    <row r="164" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="164" spans="1:14" hidden="1" x14ac:dyDescent="0.35">
       <c r="A164" t="s">
         <v>206</v>
       </c>
@@ -8720,7 +8851,7 @@
         <v>5541</v>
       </c>
     </row>
-    <row r="165" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="165" spans="1:14" hidden="1" x14ac:dyDescent="0.35">
       <c r="A165" t="s">
         <v>207</v>
       </c>
@@ -8764,7 +8895,7 @@
         <v>5541</v>
       </c>
     </row>
-    <row r="166" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="166" spans="1:14" hidden="1" x14ac:dyDescent="0.35">
       <c r="A166" t="s">
         <v>208</v>
       </c>
@@ -8808,7 +8939,7 @@
         <v>5536</v>
       </c>
     </row>
-    <row r="167" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="167" spans="1:14" hidden="1" x14ac:dyDescent="0.35">
       <c r="A167" t="s">
         <v>209</v>
       </c>
@@ -8852,7 +8983,7 @@
         <v>5536</v>
       </c>
     </row>
-    <row r="168" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="168" spans="1:14" hidden="1" x14ac:dyDescent="0.35">
       <c r="A168" t="s">
         <v>210</v>
       </c>
@@ -8896,7 +9027,7 @@
         <v>5535</v>
       </c>
     </row>
-    <row r="169" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="169" spans="1:14" hidden="1" x14ac:dyDescent="0.35">
       <c r="A169" t="s">
         <v>211</v>
       </c>
@@ -8940,7 +9071,7 @@
         <v>5535</v>
       </c>
     </row>
-    <row r="170" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="170" spans="1:14" hidden="1" x14ac:dyDescent="0.35">
       <c r="A170" t="s">
         <v>212</v>
       </c>
@@ -8984,7 +9115,7 @@
         <v>5535</v>
       </c>
     </row>
-    <row r="171" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="171" spans="1:14" hidden="1" x14ac:dyDescent="0.35">
       <c r="A171" t="s">
         <v>214</v>
       </c>
@@ -9028,7 +9159,7 @@
         <v>5535</v>
       </c>
     </row>
-    <row r="172" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="172" spans="1:14" hidden="1" x14ac:dyDescent="0.35">
       <c r="A172" t="s">
         <v>215</v>
       </c>
@@ -9072,7 +9203,7 @@
         <v>5535</v>
       </c>
     </row>
-    <row r="173" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="173" spans="1:14" hidden="1" x14ac:dyDescent="0.35">
       <c r="A173" t="s">
         <v>216</v>
       </c>
@@ -9116,7 +9247,7 @@
         <v>5535</v>
       </c>
     </row>
-    <row r="174" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="174" spans="1:14" hidden="1" x14ac:dyDescent="0.35">
       <c r="A174" t="s">
         <v>217</v>
       </c>
@@ -9160,7 +9291,7 @@
         <v>5535</v>
       </c>
     </row>
-    <row r="175" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="175" spans="1:14" hidden="1" x14ac:dyDescent="0.35">
       <c r="A175" t="s">
         <v>218</v>
       </c>
@@ -9204,7 +9335,7 @@
         <v>5535</v>
       </c>
     </row>
-    <row r="176" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="176" spans="1:14" hidden="1" x14ac:dyDescent="0.35">
       <c r="A176" t="s">
         <v>219</v>
       </c>
@@ -9248,7 +9379,7 @@
         <v>5535</v>
       </c>
     </row>
-    <row r="177" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="177" spans="1:14" hidden="1" x14ac:dyDescent="0.35">
       <c r="A177" t="s">
         <v>220</v>
       </c>
@@ -9292,7 +9423,7 @@
         <v>5535</v>
       </c>
     </row>
-    <row r="178" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="178" spans="1:14" hidden="1" x14ac:dyDescent="0.35">
       <c r="A178" t="s">
         <v>221</v>
       </c>
@@ -9336,7 +9467,7 @@
         <v>5535</v>
       </c>
     </row>
-    <row r="179" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="179" spans="1:14" hidden="1" x14ac:dyDescent="0.35">
       <c r="A179" t="s">
         <v>222</v>
       </c>
@@ -9380,7 +9511,7 @@
         <v>5535</v>
       </c>
     </row>
-    <row r="180" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="180" spans="1:14" hidden="1" x14ac:dyDescent="0.35">
       <c r="A180" t="s">
         <v>223</v>
       </c>
@@ -9424,7 +9555,7 @@
         <v>5535</v>
       </c>
     </row>
-    <row r="181" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="181" spans="1:14" hidden="1" x14ac:dyDescent="0.35">
       <c r="A181" t="s">
         <v>224</v>
       </c>
@@ -9468,7 +9599,7 @@
         <v>5535</v>
       </c>
     </row>
-    <row r="182" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="182" spans="1:14" hidden="1" x14ac:dyDescent="0.35">
       <c r="A182" t="s">
         <v>225</v>
       </c>
@@ -9512,7 +9643,7 @@
         <v>5535</v>
       </c>
     </row>
-    <row r="183" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="183" spans="1:14" hidden="1" x14ac:dyDescent="0.35">
       <c r="A183" t="s">
         <v>226</v>
       </c>
@@ -9556,7 +9687,7 @@
         <v>5535</v>
       </c>
     </row>
-    <row r="184" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="184" spans="1:14" hidden="1" x14ac:dyDescent="0.35">
       <c r="A184" t="s">
         <v>227</v>
       </c>
@@ -9600,7 +9731,7 @@
         <v>5535</v>
       </c>
     </row>
-    <row r="185" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="185" spans="1:14" hidden="1" x14ac:dyDescent="0.35">
       <c r="A185" t="s">
         <v>228</v>
       </c>
@@ -9644,7 +9775,7 @@
         <v>5535</v>
       </c>
     </row>
-    <row r="186" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="186" spans="1:14" hidden="1" x14ac:dyDescent="0.35">
       <c r="A186" t="s">
         <v>229</v>
       </c>
@@ -9688,7 +9819,7 @@
         <v>5532</v>
       </c>
     </row>
-    <row r="187" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="187" spans="1:14" hidden="1" x14ac:dyDescent="0.35">
       <c r="A187" t="s">
         <v>230</v>
       </c>
@@ -9732,7 +9863,7 @@
         <v>5532</v>
       </c>
     </row>
-    <row r="188" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="188" spans="1:14" hidden="1" x14ac:dyDescent="0.35">
       <c r="A188" t="s">
         <v>231</v>
       </c>
@@ -9776,7 +9907,7 @@
         <v>5532</v>
       </c>
     </row>
-    <row r="189" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="189" spans="1:14" hidden="1" x14ac:dyDescent="0.35">
       <c r="A189" t="s">
         <v>232</v>
       </c>
@@ -9820,7 +9951,7 @@
         <v>5532</v>
       </c>
     </row>
-    <row r="190" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="190" spans="1:14" hidden="1" x14ac:dyDescent="0.35">
       <c r="A190" t="s">
         <v>233</v>
       </c>
@@ -9864,7 +9995,7 @@
         <v>5532</v>
       </c>
     </row>
-    <row r="191" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="191" spans="1:14" hidden="1" x14ac:dyDescent="0.35">
       <c r="A191" s="1" t="s">
         <v>234</v>
       </c>
@@ -9908,7 +10039,7 @@
         <v>5532</v>
       </c>
     </row>
-    <row r="192" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="192" spans="1:14" hidden="1" x14ac:dyDescent="0.35">
       <c r="A192" t="s">
         <v>235</v>
       </c>
@@ -9952,7 +10083,7 @@
         <v>5532</v>
       </c>
     </row>
-    <row r="193" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="193" spans="1:14" hidden="1" x14ac:dyDescent="0.35">
       <c r="A193" t="s">
         <v>236</v>
       </c>
@@ -9996,7 +10127,7 @@
         <v>5532</v>
       </c>
     </row>
-    <row r="194" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="194" spans="1:14" hidden="1" x14ac:dyDescent="0.35">
       <c r="A194" t="s">
         <v>237</v>
       </c>
@@ -10040,7 +10171,7 @@
         <v>5530</v>
       </c>
     </row>
-    <row r="195" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="195" spans="1:14" hidden="1" x14ac:dyDescent="0.35">
       <c r="A195" t="s">
         <v>239</v>
       </c>
@@ -10084,7 +10215,7 @@
         <v>5530</v>
       </c>
     </row>
-    <row r="196" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="196" spans="1:14" hidden="1" x14ac:dyDescent="0.35">
       <c r="A196" t="s">
         <v>240</v>
       </c>
@@ -10128,7 +10259,7 @@
         <v>5530</v>
       </c>
     </row>
-    <row r="197" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="197" spans="1:14" hidden="1" x14ac:dyDescent="0.35">
       <c r="A197" t="s">
         <v>241</v>
       </c>
@@ -10172,7 +10303,7 @@
         <v>5530</v>
       </c>
     </row>
-    <row r="198" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="198" spans="1:14" hidden="1" x14ac:dyDescent="0.35">
       <c r="A198" t="s">
         <v>242</v>
       </c>
@@ -10216,7 +10347,7 @@
         <v>5530</v>
       </c>
     </row>
-    <row r="199" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="199" spans="1:14" hidden="1" x14ac:dyDescent="0.35">
       <c r="A199" t="s">
         <v>243</v>
       </c>
@@ -10260,7 +10391,7 @@
         <v>5530</v>
       </c>
     </row>
-    <row r="200" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="200" spans="1:14" hidden="1" x14ac:dyDescent="0.35">
       <c r="A200" t="s">
         <v>244</v>
       </c>
@@ -10304,7 +10435,7 @@
         <v>5530</v>
       </c>
     </row>
-    <row r="201" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="201" spans="1:14" hidden="1" x14ac:dyDescent="0.35">
       <c r="A201" t="s">
         <v>245</v>
       </c>
@@ -10348,7 +10479,7 @@
         <v>5530</v>
       </c>
     </row>
-    <row r="202" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="202" spans="1:14" hidden="1" x14ac:dyDescent="0.35">
       <c r="A202" t="s">
         <v>246</v>
       </c>
@@ -10392,7 +10523,7 @@
         <v>5536</v>
       </c>
     </row>
-    <row r="203" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="203" spans="1:14" hidden="1" x14ac:dyDescent="0.35">
       <c r="A203" t="s">
         <v>247</v>
       </c>
@@ -10436,7 +10567,7 @@
         <v>5536</v>
       </c>
     </row>
-    <row r="204" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="204" spans="1:14" hidden="1" x14ac:dyDescent="0.35">
       <c r="A204" t="s">
         <v>248</v>
       </c>
@@ -10480,7 +10611,7 @@
         <v>5536</v>
       </c>
     </row>
-    <row r="205" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="205" spans="1:14" hidden="1" x14ac:dyDescent="0.35">
       <c r="A205" t="s">
         <v>249</v>
       </c>
@@ -10524,7 +10655,7 @@
         <v>5536</v>
       </c>
     </row>
-    <row r="206" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="206" spans="1:14" hidden="1" x14ac:dyDescent="0.35">
       <c r="A206" t="s">
         <v>250</v>
       </c>
@@ -10568,7 +10699,7 @@
         <v>5536</v>
       </c>
     </row>
-    <row r="207" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="207" spans="1:14" hidden="1" x14ac:dyDescent="0.35">
       <c r="A207" t="s">
         <v>252</v>
       </c>
@@ -10612,7 +10743,7 @@
         <v>5536</v>
       </c>
     </row>
-    <row r="208" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="208" spans="1:14" hidden="1" x14ac:dyDescent="0.35">
       <c r="A208" t="s">
         <v>253</v>
       </c>
@@ -10656,7 +10787,7 @@
         <v>5536</v>
       </c>
     </row>
-    <row r="209" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="209" spans="1:14" hidden="1" x14ac:dyDescent="0.35">
       <c r="A209" t="s">
         <v>254</v>
       </c>
@@ -10700,7 +10831,7 @@
         <v>5536</v>
       </c>
     </row>
-    <row r="210" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="210" spans="1:14" hidden="1" x14ac:dyDescent="0.35">
       <c r="A210" t="s">
         <v>255</v>
       </c>
@@ -10744,7 +10875,7 @@
         <v>5536</v>
       </c>
     </row>
-    <row r="211" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="211" spans="1:14" hidden="1" x14ac:dyDescent="0.35">
       <c r="A211" t="s">
         <v>256</v>
       </c>
@@ -10788,7 +10919,7 @@
         <v>5536</v>
       </c>
     </row>
-    <row r="212" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="212" spans="1:14" hidden="1" x14ac:dyDescent="0.35">
       <c r="A212" t="s">
         <v>257</v>
       </c>
@@ -10832,7 +10963,7 @@
         <v>5536</v>
       </c>
     </row>
-    <row r="213" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="213" spans="1:14" hidden="1" x14ac:dyDescent="0.35">
       <c r="A213" t="s">
         <v>258</v>
       </c>
@@ -10876,7 +11007,7 @@
         <v>5536</v>
       </c>
     </row>
-    <row r="214" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="214" spans="1:14" hidden="1" x14ac:dyDescent="0.35">
       <c r="A214" t="s">
         <v>259</v>
       </c>
@@ -10920,7 +11051,7 @@
         <v>5539</v>
       </c>
     </row>
-    <row r="215" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="215" spans="1:14" hidden="1" x14ac:dyDescent="0.35">
       <c r="A215" t="s">
         <v>260</v>
       </c>
@@ -10964,7 +11095,7 @@
         <v>5539</v>
       </c>
     </row>
-    <row r="216" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="216" spans="1:14" hidden="1" x14ac:dyDescent="0.35">
       <c r="A216" t="s">
         <v>261</v>
       </c>
@@ -11008,7 +11139,7 @@
         <v>5539</v>
       </c>
     </row>
-    <row r="217" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="217" spans="1:14" hidden="1" x14ac:dyDescent="0.35">
       <c r="A217" t="s">
         <v>262</v>
       </c>
@@ -11052,7 +11183,7 @@
         <v>5539</v>
       </c>
     </row>
-    <row r="218" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="218" spans="1:14" hidden="1" x14ac:dyDescent="0.35">
       <c r="A218" t="s">
         <v>263</v>
       </c>
@@ -11096,7 +11227,7 @@
         <v>5539</v>
       </c>
     </row>
-    <row r="219" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="219" spans="1:14" hidden="1" x14ac:dyDescent="0.35">
       <c r="A219" t="s">
         <v>264</v>
       </c>
@@ -11140,7 +11271,7 @@
         <v>5539</v>
       </c>
     </row>
-    <row r="220" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="220" spans="1:14" hidden="1" x14ac:dyDescent="0.35">
       <c r="A220" t="s">
         <v>265</v>
       </c>
@@ -11184,7 +11315,7 @@
         <v>5539</v>
       </c>
     </row>
-    <row r="221" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="221" spans="1:14" hidden="1" x14ac:dyDescent="0.35">
       <c r="A221" t="s">
         <v>266</v>
       </c>
@@ -11228,7 +11359,7 @@
         <v>5539</v>
       </c>
     </row>
-    <row r="222" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="222" spans="1:14" hidden="1" x14ac:dyDescent="0.35">
       <c r="A222" t="s">
         <v>267</v>
       </c>
@@ -11272,7 +11403,7 @@
         <v>5532</v>
       </c>
     </row>
-    <row r="223" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="223" spans="1:14" hidden="1" x14ac:dyDescent="0.35">
       <c r="A223" t="s">
         <v>268</v>
       </c>
@@ -11316,7 +11447,7 @@
         <v>5532</v>
       </c>
     </row>
-    <row r="224" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="224" spans="1:14" hidden="1" x14ac:dyDescent="0.35">
       <c r="A224" t="s">
         <v>269</v>
       </c>
@@ -11360,7 +11491,7 @@
         <v>5535</v>
       </c>
     </row>
-    <row r="225" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="225" spans="1:14" hidden="1" x14ac:dyDescent="0.35">
       <c r="A225" t="s">
         <v>270</v>
       </c>
@@ -11404,7 +11535,7 @@
         <v>5535</v>
       </c>
     </row>
-    <row r="226" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="226" spans="1:14" hidden="1" x14ac:dyDescent="0.35">
       <c r="A226" t="s">
         <v>271</v>
       </c>
@@ -11448,7 +11579,7 @@
         <v>5535</v>
       </c>
     </row>
-    <row r="227" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="227" spans="1:14" hidden="1" x14ac:dyDescent="0.35">
       <c r="A227" t="s">
         <v>272</v>
       </c>
@@ -11492,7 +11623,7 @@
         <v>5535</v>
       </c>
     </row>
-    <row r="228" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="228" spans="1:14" hidden="1" x14ac:dyDescent="0.35">
       <c r="A228" t="s">
         <v>273</v>
       </c>
@@ -11536,7 +11667,7 @@
         <v>5535</v>
       </c>
     </row>
-    <row r="229" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="229" spans="1:14" hidden="1" x14ac:dyDescent="0.35">
       <c r="A229" t="s">
         <v>274</v>
       </c>
@@ -11580,7 +11711,7 @@
         <v>5535</v>
       </c>
     </row>
-    <row r="230" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="230" spans="1:14" hidden="1" x14ac:dyDescent="0.35">
       <c r="A230" t="s">
         <v>275</v>
       </c>
@@ -11624,7 +11755,7 @@
         <v>5530</v>
       </c>
     </row>
-    <row r="231" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="231" spans="1:14" hidden="1" x14ac:dyDescent="0.35">
       <c r="A231" t="s">
         <v>277</v>
       </c>
@@ -11668,7 +11799,7 @@
         <v>5530</v>
       </c>
     </row>
-    <row r="232" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="232" spans="1:14" hidden="1" x14ac:dyDescent="0.35">
       <c r="A232" t="s">
         <v>278</v>
       </c>
@@ -11712,7 +11843,7 @@
         <v>5530</v>
       </c>
     </row>
-    <row r="233" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="233" spans="1:14" hidden="1" x14ac:dyDescent="0.35">
       <c r="A233" t="s">
         <v>279</v>
       </c>
@@ -11756,7 +11887,7 @@
         <v>5530</v>
       </c>
     </row>
-    <row r="234" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="234" spans="1:14" hidden="1" x14ac:dyDescent="0.35">
       <c r="A234" t="s">
         <v>280</v>
       </c>
@@ -11800,7 +11931,7 @@
         <v>5530</v>
       </c>
     </row>
-    <row r="235" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="235" spans="1:14" hidden="1" x14ac:dyDescent="0.35">
       <c r="A235" t="s">
         <v>281</v>
       </c>
@@ -11844,7 +11975,7 @@
         <v>5530</v>
       </c>
     </row>
-    <row r="236" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="236" spans="1:14" hidden="1" x14ac:dyDescent="0.35">
       <c r="A236" t="s">
         <v>282</v>
       </c>
@@ -11888,7 +12019,7 @@
         <v>5530</v>
       </c>
     </row>
-    <row r="237" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="237" spans="1:14" hidden="1" x14ac:dyDescent="0.35">
       <c r="A237" t="s">
         <v>283</v>
       </c>
@@ -11932,7 +12063,7 @@
         <v>5530</v>
       </c>
     </row>
-    <row r="238" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="238" spans="1:14" hidden="1" x14ac:dyDescent="0.35">
       <c r="A238" t="s">
         <v>284</v>
       </c>
@@ -11976,7 +12107,7 @@
         <v>5530</v>
       </c>
     </row>
-    <row r="239" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="239" spans="1:14" hidden="1" x14ac:dyDescent="0.35">
       <c r="A239" t="s">
         <v>285</v>
       </c>
@@ -12020,7 +12151,7 @@
         <v>5530</v>
       </c>
     </row>
-    <row r="240" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="240" spans="1:14" hidden="1" x14ac:dyDescent="0.35">
       <c r="A240" t="s">
         <v>286</v>
       </c>
@@ -12064,7 +12195,7 @@
         <v>5530</v>
       </c>
     </row>
-    <row r="241" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="241" spans="1:14" hidden="1" x14ac:dyDescent="0.35">
       <c r="A241" t="s">
         <v>287</v>
       </c>
@@ -12108,7 +12239,7 @@
         <v>5530</v>
       </c>
     </row>
-    <row r="242" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="242" spans="1:14" hidden="1" x14ac:dyDescent="0.35">
       <c r="A242" t="s">
         <v>288</v>
       </c>
@@ -12152,7 +12283,7 @@
         <v>5530</v>
       </c>
     </row>
-    <row r="243" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="243" spans="1:14" hidden="1" x14ac:dyDescent="0.35">
       <c r="A243" t="s">
         <v>289</v>
       </c>
@@ -12196,7 +12327,7 @@
         <v>5530</v>
       </c>
     </row>
-    <row r="244" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="244" spans="1:14" hidden="1" x14ac:dyDescent="0.35">
       <c r="A244" t="s">
         <v>290</v>
       </c>
@@ -12240,7 +12371,7 @@
         <v>5532</v>
       </c>
     </row>
-    <row r="245" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="245" spans="1:14" hidden="1" x14ac:dyDescent="0.35">
       <c r="A245" t="s">
         <v>291</v>
       </c>
@@ -12284,7 +12415,7 @@
         <v>5532</v>
       </c>
     </row>
-    <row r="246" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="246" spans="1:14" hidden="1" x14ac:dyDescent="0.35">
       <c r="A246" t="s">
         <v>292</v>
       </c>
@@ -12328,7 +12459,7 @@
         <v>5532</v>
       </c>
     </row>
-    <row r="247" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="247" spans="1:14" hidden="1" x14ac:dyDescent="0.35">
       <c r="A247" t="s">
         <v>293</v>
       </c>
@@ -12372,7 +12503,7 @@
         <v>5532</v>
       </c>
     </row>
-    <row r="248" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="248" spans="1:14" hidden="1" x14ac:dyDescent="0.35">
       <c r="A248" t="s">
         <v>294</v>
       </c>
@@ -12416,7 +12547,7 @@
         <v>5532</v>
       </c>
     </row>
-    <row r="249" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="249" spans="1:14" hidden="1" x14ac:dyDescent="0.35">
       <c r="A249" t="s">
         <v>295</v>
       </c>
@@ -12460,7 +12591,7 @@
         <v>5532</v>
       </c>
     </row>
-    <row r="250" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="250" spans="1:14" hidden="1" x14ac:dyDescent="0.35">
       <c r="A250" t="s">
         <v>296</v>
       </c>
@@ -12504,7 +12635,7 @@
         <v>5532</v>
       </c>
     </row>
-    <row r="251" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="251" spans="1:14" hidden="1" x14ac:dyDescent="0.35">
       <c r="A251" t="s">
         <v>297</v>
       </c>
@@ -12548,7 +12679,7 @@
         <v>5532</v>
       </c>
     </row>
-    <row r="252" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="252" spans="1:14" hidden="1" x14ac:dyDescent="0.35">
       <c r="A252" t="s">
         <v>298</v>
       </c>
@@ -12592,7 +12723,7 @@
         <v>5535</v>
       </c>
     </row>
-    <row r="253" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="253" spans="1:14" hidden="1" x14ac:dyDescent="0.35">
       <c r="A253" t="s">
         <v>299</v>
       </c>
@@ -12636,7 +12767,7 @@
         <v>5535</v>
       </c>
     </row>
-    <row r="254" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="254" spans="1:14" hidden="1" x14ac:dyDescent="0.35">
       <c r="A254" t="s">
         <v>300</v>
       </c>
@@ -12680,7 +12811,7 @@
         <v>5535</v>
       </c>
     </row>
-    <row r="255" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="255" spans="1:14" hidden="1" x14ac:dyDescent="0.35">
       <c r="A255" t="s">
         <v>301</v>
       </c>
@@ -12724,7 +12855,7 @@
         <v>5535</v>
       </c>
     </row>
-    <row r="256" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="256" spans="1:14" hidden="1" x14ac:dyDescent="0.35">
       <c r="A256" t="s">
         <v>302</v>
       </c>
@@ -12768,7 +12899,7 @@
         <v>5535</v>
       </c>
     </row>
-    <row r="257" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="257" spans="1:14" hidden="1" x14ac:dyDescent="0.35">
       <c r="A257" t="s">
         <v>303</v>
       </c>
@@ -12812,7 +12943,7 @@
         <v>5535</v>
       </c>
     </row>
-    <row r="258" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="258" spans="1:14" hidden="1" x14ac:dyDescent="0.35">
       <c r="A258" t="s">
         <v>304</v>
       </c>
@@ -12856,7 +12987,7 @@
         <v>5535</v>
       </c>
     </row>
-    <row r="259" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="259" spans="1:14" hidden="1" x14ac:dyDescent="0.35">
       <c r="A259" t="s">
         <v>305</v>
       </c>
@@ -12900,7 +13031,7 @@
         <v>5535</v>
       </c>
     </row>
-    <row r="260" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="260" spans="1:14" hidden="1" x14ac:dyDescent="0.35">
       <c r="A260" t="s">
         <v>306</v>
       </c>
@@ -12944,7 +13075,7 @@
         <v>5536</v>
       </c>
     </row>
-    <row r="261" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="261" spans="1:14" hidden="1" x14ac:dyDescent="0.35">
       <c r="A261" t="s">
         <v>307</v>
       </c>
@@ -12988,7 +13119,7 @@
         <v>5536</v>
       </c>
     </row>
-    <row r="262" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="262" spans="1:14" hidden="1" x14ac:dyDescent="0.35">
       <c r="A262" t="s">
         <v>308</v>
       </c>
@@ -13032,7 +13163,7 @@
         <v>5536</v>
       </c>
     </row>
-    <row r="263" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="263" spans="1:14" hidden="1" x14ac:dyDescent="0.35">
       <c r="A263" t="s">
         <v>309</v>
       </c>
@@ -13076,7 +13207,7 @@
         <v>5536</v>
       </c>
     </row>
-    <row r="264" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="264" spans="1:14" hidden="1" x14ac:dyDescent="0.35">
       <c r="A264" t="s">
         <v>310</v>
       </c>
@@ -13120,7 +13251,7 @@
         <v>5536</v>
       </c>
     </row>
-    <row r="265" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="265" spans="1:14" hidden="1" x14ac:dyDescent="0.35">
       <c r="A265" t="s">
         <v>311</v>
       </c>
@@ -13164,7 +13295,7 @@
         <v>5536</v>
       </c>
     </row>
-    <row r="266" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="266" spans="1:14" hidden="1" x14ac:dyDescent="0.35">
       <c r="A266" t="s">
         <v>312</v>
       </c>
@@ -13208,7 +13339,7 @@
         <v>5536</v>
       </c>
     </row>
-    <row r="267" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="267" spans="1:14" hidden="1" x14ac:dyDescent="0.35">
       <c r="A267" t="s">
         <v>314</v>
       </c>
@@ -13252,7 +13383,7 @@
         <v>5536</v>
       </c>
     </row>
-    <row r="268" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="268" spans="1:14" hidden="1" x14ac:dyDescent="0.35">
       <c r="A268" t="s">
         <v>315</v>
       </c>
@@ -13296,7 +13427,7 @@
         <v>5536</v>
       </c>
     </row>
-    <row r="269" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="269" spans="1:14" hidden="1" x14ac:dyDescent="0.35">
       <c r="A269" t="s">
         <v>316</v>
       </c>
@@ -13340,7 +13471,7 @@
         <v>5536</v>
       </c>
     </row>
-    <row r="270" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="270" spans="1:14" hidden="1" x14ac:dyDescent="0.35">
       <c r="A270" t="s">
         <v>317</v>
       </c>
@@ -13384,7 +13515,7 @@
         <v>5540</v>
       </c>
     </row>
-    <row r="271" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="271" spans="1:14" hidden="1" x14ac:dyDescent="0.35">
       <c r="A271" t="s">
         <v>318</v>
       </c>
@@ -13428,7 +13559,7 @@
         <v>5540</v>
       </c>
     </row>
-    <row r="272" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="272" spans="1:14" hidden="1" x14ac:dyDescent="0.35">
       <c r="A272" t="s">
         <v>319</v>
       </c>
@@ -13472,7 +13603,7 @@
         <v>5543</v>
       </c>
     </row>
-    <row r="273" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="273" spans="1:14" hidden="1" x14ac:dyDescent="0.35">
       <c r="A273" t="s">
         <v>320</v>
       </c>
@@ -13516,7 +13647,7 @@
         <v>5543</v>
       </c>
     </row>
-    <row r="274" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="274" spans="1:14" hidden="1" x14ac:dyDescent="0.35">
       <c r="A274" t="s">
         <v>321</v>
       </c>
@@ -13560,7 +13691,7 @@
         <v>5543</v>
       </c>
     </row>
-    <row r="275" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="275" spans="1:14" hidden="1" x14ac:dyDescent="0.35">
       <c r="A275" t="s">
         <v>322</v>
       </c>
@@ -13604,7 +13735,7 @@
         <v>5543</v>
       </c>
     </row>
-    <row r="276" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="276" spans="1:14" hidden="1" x14ac:dyDescent="0.35">
       <c r="A276" t="s">
         <v>323</v>
       </c>
@@ -13648,7 +13779,7 @@
         <v>5543</v>
       </c>
     </row>
-    <row r="277" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="277" spans="1:14" hidden="1" x14ac:dyDescent="0.35">
       <c r="A277" t="s">
         <v>324</v>
       </c>
@@ -13692,7 +13823,7 @@
         <v>5543</v>
       </c>
     </row>
-    <row r="278" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="278" spans="1:14" hidden="1" x14ac:dyDescent="0.35">
       <c r="A278" t="s">
         <v>325</v>
       </c>
@@ -13736,7 +13867,7 @@
         <v>5541</v>
       </c>
     </row>
-    <row r="279" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="279" spans="1:14" hidden="1" x14ac:dyDescent="0.35">
       <c r="A279" t="s">
         <v>326</v>
       </c>
@@ -13780,7 +13911,7 @@
         <v>5541</v>
       </c>
     </row>
-    <row r="280" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="280" spans="1:14" hidden="1" x14ac:dyDescent="0.35">
       <c r="A280" t="s">
         <v>327</v>
       </c>
@@ -13824,7 +13955,7 @@
         <v>5541</v>
       </c>
     </row>
-    <row r="281" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="281" spans="1:14" hidden="1" x14ac:dyDescent="0.35">
       <c r="A281" t="s">
         <v>328</v>
       </c>
@@ -13868,7 +13999,7 @@
         <v>5541</v>
       </c>
     </row>
-    <row r="282" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="282" spans="1:14" hidden="1" x14ac:dyDescent="0.35">
       <c r="A282" t="s">
         <v>329</v>
       </c>
@@ -13912,7 +14043,7 @@
         <v>5541</v>
       </c>
     </row>
-    <row r="283" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="283" spans="1:14" hidden="1" x14ac:dyDescent="0.35">
       <c r="A283" t="s">
         <v>330</v>
       </c>
@@ -13956,7 +14087,7 @@
         <v>5541</v>
       </c>
     </row>
-    <row r="284" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="284" spans="1:14" hidden="1" x14ac:dyDescent="0.35">
       <c r="A284" t="s">
         <v>331</v>
       </c>
@@ -14000,7 +14131,7 @@
         <v>5535</v>
       </c>
     </row>
-    <row r="285" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="285" spans="1:14" hidden="1" x14ac:dyDescent="0.35">
       <c r="A285" t="s">
         <v>332</v>
       </c>
@@ -14044,7 +14175,7 @@
         <v>5535</v>
       </c>
     </row>
-    <row r="286" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="286" spans="1:14" hidden="1" x14ac:dyDescent="0.35">
       <c r="A286" t="s">
         <v>333</v>
       </c>
@@ -14088,7 +14219,7 @@
         <v>5535</v>
       </c>
     </row>
-    <row r="287" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="287" spans="1:14" hidden="1" x14ac:dyDescent="0.35">
       <c r="A287" t="s">
         <v>334</v>
       </c>
@@ -14132,7 +14263,7 @@
         <v>5535</v>
       </c>
     </row>
-    <row r="288" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="288" spans="1:14" hidden="1" x14ac:dyDescent="0.35">
       <c r="A288" t="s">
         <v>335</v>
       </c>
@@ -14176,7 +14307,7 @@
         <v>5535</v>
       </c>
     </row>
-    <row r="289" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="289" spans="1:14" hidden="1" x14ac:dyDescent="0.35">
       <c r="A289" t="s">
         <v>336</v>
       </c>
@@ -14220,7 +14351,7 @@
         <v>5535</v>
       </c>
     </row>
-    <row r="290" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="290" spans="1:14" hidden="1" x14ac:dyDescent="0.35">
       <c r="A290" t="s">
         <v>337</v>
       </c>
@@ -14264,7 +14395,7 @@
         <v>5536</v>
       </c>
     </row>
-    <row r="291" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="291" spans="1:14" hidden="1" x14ac:dyDescent="0.35">
       <c r="A291" t="s">
         <v>339</v>
       </c>
@@ -14308,7 +14439,7 @@
         <v>5536</v>
       </c>
     </row>
-    <row r="292" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="292" spans="1:14" hidden="1" x14ac:dyDescent="0.35">
       <c r="A292" t="s">
         <v>340</v>
       </c>
@@ -14352,7 +14483,7 @@
         <v>5536</v>
       </c>
     </row>
-    <row r="293" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="293" spans="1:14" hidden="1" x14ac:dyDescent="0.35">
       <c r="A293" t="s">
         <v>341</v>
       </c>
@@ -14396,7 +14527,7 @@
         <v>5536</v>
       </c>
     </row>
-    <row r="294" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="294" spans="1:14" hidden="1" x14ac:dyDescent="0.35">
       <c r="A294" t="s">
         <v>342</v>
       </c>
@@ -14440,7 +14571,7 @@
         <v>5536</v>
       </c>
     </row>
-    <row r="295" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="295" spans="1:14" hidden="1" x14ac:dyDescent="0.35">
       <c r="A295" t="s">
         <v>343</v>
       </c>
@@ -14484,7 +14615,7 @@
         <v>5536</v>
       </c>
     </row>
-    <row r="296" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="296" spans="1:14" hidden="1" x14ac:dyDescent="0.35">
       <c r="A296" t="s">
         <v>344</v>
       </c>
@@ -14528,7 +14659,7 @@
         <v>5535</v>
       </c>
     </row>
-    <row r="297" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="297" spans="1:14" hidden="1" x14ac:dyDescent="0.35">
       <c r="A297" t="s">
         <v>345</v>
       </c>
@@ -14572,7 +14703,7 @@
         <v>5535</v>
       </c>
     </row>
-    <row r="298" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="298" spans="1:14" hidden="1" x14ac:dyDescent="0.35">
       <c r="A298" t="s">
         <v>346</v>
       </c>
@@ -14616,7 +14747,7 @@
         <v>5535</v>
       </c>
     </row>
-    <row r="299" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="299" spans="1:14" hidden="1" x14ac:dyDescent="0.35">
       <c r="A299" t="s">
         <v>347</v>
       </c>
@@ -14660,7 +14791,7 @@
         <v>5535</v>
       </c>
     </row>
-    <row r="300" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="300" spans="1:14" hidden="1" x14ac:dyDescent="0.35">
       <c r="A300" t="s">
         <v>348</v>
       </c>
@@ -14704,7 +14835,7 @@
         <v>5535</v>
       </c>
     </row>
-    <row r="301" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="301" spans="1:14" hidden="1" x14ac:dyDescent="0.35">
       <c r="A301" t="s">
         <v>349</v>
       </c>
@@ -14748,7 +14879,7 @@
         <v>5535</v>
       </c>
     </row>
-    <row r="302" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="302" spans="1:14" hidden="1" x14ac:dyDescent="0.35">
       <c r="A302" t="s">
         <v>350</v>
       </c>
@@ -14792,7 +14923,7 @@
         <v>5535</v>
       </c>
     </row>
-    <row r="303" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="303" spans="1:14" hidden="1" x14ac:dyDescent="0.35">
       <c r="A303" t="s">
         <v>351</v>
       </c>
@@ -14836,7 +14967,7 @@
         <v>5535</v>
       </c>
     </row>
-    <row r="304" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="304" spans="1:14" hidden="1" x14ac:dyDescent="0.35">
       <c r="A304" t="s">
         <v>352</v>
       </c>
@@ -14880,7 +15011,7 @@
         <v>5539</v>
       </c>
     </row>
-    <row r="305" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="305" spans="1:14" hidden="1" x14ac:dyDescent="0.35">
       <c r="A305" t="s">
         <v>353</v>
       </c>
@@ -14924,7 +15055,7 @@
         <v>5539</v>
       </c>
     </row>
-    <row r="306" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="306" spans="1:14" hidden="1" x14ac:dyDescent="0.35">
       <c r="A306" t="s">
         <v>354</v>
       </c>
@@ -14968,7 +15099,7 @@
         <v>5539</v>
       </c>
     </row>
-    <row r="307" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="307" spans="1:14" hidden="1" x14ac:dyDescent="0.35">
       <c r="A307" t="s">
         <v>355</v>
       </c>
@@ -15012,7 +15143,7 @@
         <v>5539</v>
       </c>
     </row>
-    <row r="308" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="308" spans="1:14" hidden="1" x14ac:dyDescent="0.35">
       <c r="A308" t="s">
         <v>356</v>
       </c>
@@ -15056,7 +15187,7 @@
         <v>5539</v>
       </c>
     </row>
-    <row r="309" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="309" spans="1:14" hidden="1" x14ac:dyDescent="0.35">
       <c r="A309" t="s">
         <v>357</v>
       </c>
@@ -15100,7 +15231,7 @@
         <v>5539</v>
       </c>
     </row>
-    <row r="310" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="310" spans="1:14" hidden="1" x14ac:dyDescent="0.35">
       <c r="A310" t="s">
         <v>358</v>
       </c>
@@ -15144,7 +15275,7 @@
         <v>5539</v>
       </c>
     </row>
-    <row r="311" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="311" spans="1:14" hidden="1" x14ac:dyDescent="0.35">
       <c r="A311" t="s">
         <v>359</v>
       </c>
@@ -15186,6 +15317,106 @@
       </c>
       <c r="N311">
         <v>5539</v>
+      </c>
+    </row>
+    <row r="317" spans="1:14" ht="29" x14ac:dyDescent="0.35">
+      <c r="A317" s="6" t="s">
+        <v>360</v>
+      </c>
+      <c r="B317" s="8" t="s">
+        <v>361</v>
+      </c>
+      <c r="C317" s="10" t="s">
+        <v>362</v>
+      </c>
+      <c r="D317" s="11" t="s">
+        <v>363</v>
+      </c>
+      <c r="E317" s="12" t="s">
+        <v>364</v>
+      </c>
+      <c r="F317" s="12" t="s">
+        <v>365</v>
+      </c>
+      <c r="G317" s="10" t="s">
+        <v>366</v>
+      </c>
+      <c r="H317" s="10" t="s">
+        <v>367</v>
+      </c>
+      <c r="I317" s="13" t="s">
+        <v>368</v>
+      </c>
+      <c r="J317" s="14" t="s">
+        <v>369</v>
+      </c>
+      <c r="K317" s="4" t="s">
+        <v>370</v>
+      </c>
+      <c r="L317" s="3" t="s">
+        <v>371</v>
+      </c>
+      <c r="M317" s="3" t="s">
+        <v>372</v>
+      </c>
+      <c r="N317" s="5" t="s">
+        <v>373</v>
+      </c>
+    </row>
+    <row r="318" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="A318" s="7"/>
+      <c r="B318" s="9"/>
+      <c r="C318" s="7"/>
+      <c r="D318" s="9"/>
+      <c r="E318" s="7"/>
+      <c r="F318" s="7"/>
+      <c r="G318" s="9"/>
+      <c r="H318" s="9"/>
+      <c r="I318" s="15"/>
+      <c r="J318" s="16"/>
+    </row>
+    <row r="319" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="A319" s="7" t="s">
+        <v>0</v>
+      </c>
+      <c r="B319" s="9" t="s">
+        <v>1</v>
+      </c>
+      <c r="C319" s="7" t="s">
+        <v>2</v>
+      </c>
+      <c r="D319" s="9" t="s">
+        <v>3</v>
+      </c>
+      <c r="E319" s="7" t="s">
+        <v>4</v>
+      </c>
+      <c r="F319" s="7" t="s">
+        <v>5</v>
+      </c>
+      <c r="G319" s="9" t="s">
+        <v>6</v>
+      </c>
+      <c r="H319" s="9" t="s">
+        <v>7</v>
+      </c>
+      <c r="I319" s="15" t="s">
+        <v>8</v>
+      </c>
+      <c r="J319" s="16" t="s">
+        <v>9</v>
+      </c>
+      <c r="K319" t="s">
+        <v>10</v>
+      </c>
+      <c r="L319" t="s">
+        <v>11</v>
+      </c>
+      <c r="M319" t="s">
+        <v>10</v>
+      </c>
+      <c r="N319" t="s">
+        <v>12</v>
       </c>
     </row>
   </sheetData>

</xml_diff>